<commit_message>
Corrected the table. Next step would be to see if the random forrest can be boosted using XGBoost.
</commit_message>
<xml_diff>
--- a/result_table.xlsx
+++ b/result_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Housing-Prices\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D8AD867-AB7B-4242-9C9E-4B7687522BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{499E0206-49E8-4058-AB92-A86492F7F94A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-83" yWindow="0" windowWidth="10965" windowHeight="12863" xr2:uid="{A1F1EF00-C3AB-4D9B-91EC-3DF2E2D3820D}"/>
   </bookViews>
@@ -125,12 +125,21 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -151,8 +160,8 @@
     <tableColumn id="2" xr3:uid="{FB8DD280-3656-45C3-B3CA-89D84BCE223E}" name="Scaling"/>
     <tableColumn id="3" xr3:uid="{13E2FC1D-A2E8-4A00-BD90-83F6756268DC}" name="Removing columns where #NaN &gt; 90%"/>
     <tableColumn id="4" xr3:uid="{7EB146EE-B238-4F48-ADE2-2BC2C2ECEB79}" name="RMSE"/>
-    <tableColumn id="5" xr3:uid="{7E6B41D6-390F-4A68-8071-3542213904BB}" name="Cross Validation mean"/>
-    <tableColumn id="6" xr3:uid="{916BF664-E7E0-4AF7-AE14-F752E747B846}" name="Cross Validation std"/>
+    <tableColumn id="5" xr3:uid="{7E6B41D6-390F-4A68-8071-3542213904BB}" name="Cross Validation mean" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{916BF664-E7E0-4AF7-AE14-F752E747B846}" name="Cross Validation std" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight6" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -480,8 +489,8 @@
   <cols>
     <col min="1" max="2" width="16.06640625" customWidth="1"/>
     <col min="3" max="3" width="32.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.73046875" customWidth="1"/>
-    <col min="6" max="6" width="19.86328125" customWidth="1"/>
+    <col min="5" max="5" width="20.73046875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="19.86328125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.45">
@@ -497,10 +506,10 @@
       <c r="D1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
     </row>
@@ -517,10 +526,10 @@
       <c r="D2">
         <v>29676.115000000002</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -537,10 +546,10 @@
       <c r="D3">
         <v>29833.273000000001</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>0.755</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>6.4000000000000001E-2</v>
       </c>
     </row>
@@ -557,10 +566,10 @@
       <c r="D4">
         <v>53684770188869.398</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -577,10 +586,10 @@
       <c r="D5">
         <v>29833.273000000001</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="2">
         <v>0.80600000000000005</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="2">
         <v>6.0999999999999999E-2</v>
       </c>
     </row>
@@ -597,10 +606,10 @@
       <c r="D6">
         <v>29837.517</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="2">
         <v>0.80600000000000005</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="2">
         <v>6.9000000000000006E-2</v>
       </c>
     </row>
@@ -617,10 +626,10 @@
       <c r="D7">
         <v>29359.474999999999</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="2">
         <v>0.80400000000000005</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
         <v>8.1000000000000003E-2</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -659,7 +668,7 @@
       <c r="E8" s="2">
         <v>0.83499999999999996</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="2">
         <v>5.0999999999999997E-2</v>
       </c>
     </row>
@@ -676,10 +685,10 @@
       <c r="D9">
         <v>29193.406999999999</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="2">
         <v>0.84099999999999997</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="2">
         <v>4.2999999999999997E-2</v>
       </c>
     </row>
@@ -696,10 +705,10 @@
       <c r="D10">
         <v>28223.554</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="2">
         <v>0.84499999999999997</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="2">
         <v>4.1000000000000002E-2</v>
       </c>
       <c r="G10" s="1" t="s">

</xml_diff>